<commit_message>
Dify v3: implement all pending fixes (#11-#19)
- #14: Ambiguity Checker uses conversation_id instead of inline entities
- #15: Add org_name conversation variable + assigner node
- #17: Remove auth header from store-entities and ambiguity-checker
- #19: Enrich Upload Done answer with Avni URL and next steps
- #13: Human-input No path → corrections-prompt-answer node
- #12: 401/400/403/404/500 error handling after Download and Upload HTTP nodes
- #18: Progress answer nodes (Generating Spec, Downloading Bundle, Uploading Bundle)
- #11: PEV self-healing loop — Check Bundle/Error Verdict, Increment Retry, Save Retry Count, Check Max Retries (3), Max Retries Exhausted, Upload Error Report
- #16: Delete-config path — DELETE_CONFIG Orchestrator route, confirmation human-input, HTTP DELETE /api/implementation, success/failure/cancelled answers

All 80 edge references validated against 76 node definitions."
</commit_message>
<xml_diff>
--- a/tests/resources/scoping/Durga India Modelling.xlsx
+++ b/tests/resources/scoping/Durga India Modelling.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="58">
   <si>
     <t>Scoping</t>
   </si>
@@ -40,18 +40,6 @@
   </si>
   <si>
     <t>Not in Scope</t>
-  </si>
-  <si>
-    <t>Estimate</t>
-  </si>
-  <si>
-    <t>Durga India Estimation - 13.01.2026</t>
-  </si>
-  <si>
-    <t>Proposal</t>
-  </si>
-  <si>
-    <t>Durga India Proposal - 13.01.2026</t>
   </si>
   <si>
     <t>Location Type</t>
@@ -208,7 +196,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -219,10 +207,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -346,7 +330,7 @@
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -355,82 +339,82 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="3" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="3" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="3" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="3" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -1067,12 +1051,8 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="5"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1099,12 +1079,8 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="6"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -28939,12 +28915,10 @@
     <hyperlink r:id="rId1" location="gid=565705303" ref="B2"/>
     <hyperlink display="Durga India Modelling" location="'Location Hierarchy '!A1" ref="B3"/>
     <hyperlink r:id="rId2" location="gid=802083530" ref="B4"/>
-    <hyperlink r:id="rId3" location="gid=1556094995" ref="B6"/>
-    <hyperlink r:id="rId4" ref="B7"/>
   </hyperlinks>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -28961,26 +28935,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -29000,28 +28974,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="H1" s="11" t="s">
         <v>21</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>25</v>
       </c>
       <c r="I1" s="12"/>
       <c r="J1" s="12"/>
@@ -29044,42 +29018,42 @@
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E2" s="14"/>
       <c r="F2" s="14"/>
       <c r="G2" s="15"/>
       <c r="H2" s="11" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="14"/>
       <c r="G3" s="15"/>
       <c r="H3" s="11" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -29103,28 +29077,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="G1" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="H1" s="16" t="s">
         <v>33</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" s="16" t="s">
-        <v>37</v>
       </c>
       <c r="I1" s="12"/>
       <c r="J1" s="12"/>
@@ -29182,34 +29156,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="F1" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="G1" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="H1" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="H1" s="18" t="s">
-        <v>45</v>
-      </c>
       <c r="I1" s="18" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J1" s="18" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="K1" s="20"/>
       <c r="L1" s="12"/>
@@ -29233,20 +29207,20 @@
     </row>
     <row r="2">
       <c r="A2" s="21" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G2" s="25"/>
       <c r="H2" s="25"/>
@@ -29256,18 +29230,18 @@
     </row>
     <row r="3">
       <c r="A3" s="21" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C3" s="27"/>
       <c r="D3" s="23" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E3" s="21"/>
       <c r="F3" s="24" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G3" s="25"/>
       <c r="H3" s="25"/>
@@ -29277,23 +29251,23 @@
     </row>
     <row r="4">
       <c r="A4" s="21" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C4" s="27"/>
       <c r="D4" s="23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H4" s="25"/>
       <c r="I4" s="25"/>
@@ -29302,18 +29276,18 @@
     </row>
     <row r="5">
       <c r="A5" s="21" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C5" s="27"/>
       <c r="D5" s="23" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E5" s="21"/>
       <c r="F5" s="24" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G5" s="25"/>
       <c r="H5" s="25"/>
@@ -29323,23 +29297,23 @@
     </row>
     <row r="6">
       <c r="A6" s="21" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C6" s="27"/>
       <c r="D6" s="23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H6" s="25"/>
       <c r="I6" s="25"/>
@@ -29348,18 +29322,18 @@
     </row>
     <row r="7">
       <c r="A7" s="21" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C7" s="27"/>
       <c r="D7" s="23" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E7" s="21"/>
       <c r="F7" s="24" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G7" s="28"/>
       <c r="H7" s="25"/>
@@ -29369,18 +29343,18 @@
     </row>
     <row r="8">
       <c r="A8" s="21" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C8" s="27"/>
       <c r="D8" s="23" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E8" s="21"/>
       <c r="F8" s="24" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G8" s="28"/>
       <c r="H8" s="25"/>
@@ -29419,31 +29393,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="C1" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" s="30" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="30" t="s">
-        <v>42</v>
-      </c>
       <c r="G1" s="31" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H1" s="31" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="I1" s="31" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J1" s="12"/>
       <c r="K1" s="12"/>

</xml_diff>